<commit_message>
Add net-payable preservation proof to salary summary (Original NETPAYABLE + NET delta)
Insert ORIGINAL NETPAYABLE and NET delta (Orig-Revised) columns after REVISED
NET PAYABLE in Monthly_Summary. Confirms the sacrosanct golden rule: revised
net payable equals original net payable to the rupee (delta = Rs.0) for all 12
months and the FY total (Rs.293,29,89,494). Updates xlsx, CSV, README.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rxz8VcCB74nG7vtiLVCEGq
</commit_message>
<xml_diff>
--- a/docs/salary-monthly-summary-fy2025-26/Monthly_Salary_Deductions_Summary_FY2025-26.xlsx
+++ b/docs/salary-monthly-summary-fy2025-26/Monthly_Salary_Deductions_Summary_FY2025-26.xlsx
@@ -40,7 +40,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +50,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -84,15 +89,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK14"/>
+  <dimension ref="A1:AM14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -489,15 +495,17 @@
     <col width="24" customWidth="1" min="26" max="26"/>
     <col width="24" customWidth="1" min="27" max="27"/>
     <col width="21" customWidth="1" min="28" max="28"/>
-    <col width="12" customWidth="1" min="29" max="29"/>
-    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="21" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="24" customWidth="1" min="32" max="32"/>
-    <col width="23" customWidth="1" min="33" max="33"/>
-    <col width="22" customWidth="1" min="34" max="34"/>
-    <col width="24" customWidth="1" min="35" max="35"/>
-    <col width="24" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="24" customWidth="1" min="34" max="34"/>
+    <col width="23" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="36" max="36"/>
     <col width="24" customWidth="1" min="37" max="37"/>
+    <col width="24" customWidth="1" min="38" max="38"/>
+    <col width="24" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -643,45 +651,55 @@
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
+          <t>ORIGINAL NETPAYABLE</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>NET Δ (ORIG-REVISED)</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
           <t>OT AMOUNT</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>OT ESIC</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>NET OT</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>FESTIVAL HOLIDAY AMOUNT</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>FESTIVAL HOLIDAY ESIC</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>FESTIVAL HOLIDAY NET</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>NATIONAL/PAID HOLIDAY AMOUNT</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>NATIONAL/PAID HOLIDAY ESIC</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>NATIONAL/PAID HOLIDAY NET</t>
         </is>
@@ -775,30 +793,36 @@
         <v>229689886</v>
       </c>
       <c r="AC2" s="3" t="n">
+        <v>229689886</v>
+      </c>
+      <c r="AD2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="3" t="n">
         <v>8659813</v>
       </c>
-      <c r="AD2" s="3" t="n">
+      <c r="AF2" s="3" t="n">
         <v>50363</v>
       </c>
-      <c r="AE2" s="3" t="n">
+      <c r="AG2" s="3" t="n">
         <v>8609450</v>
       </c>
-      <c r="AF2" s="3" t="n">
+      <c r="AH2" s="3" t="n">
         <v>380478</v>
       </c>
-      <c r="AG2" s="3" t="n">
+      <c r="AI2" s="3" t="n">
         <v>2053</v>
       </c>
-      <c r="AH2" s="3" t="n">
+      <c r="AJ2" s="3" t="n">
         <v>378425</v>
       </c>
-      <c r="AI2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ2" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="AK2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM2" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -890,30 +914,36 @@
         <v>232102234</v>
       </c>
       <c r="AC3" s="3" t="n">
+        <v>232102234</v>
+      </c>
+      <c r="AD3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="3" t="n">
         <v>10285500</v>
       </c>
-      <c r="AD3" s="3" t="n">
+      <c r="AF3" s="3" t="n">
         <v>59464</v>
       </c>
-      <c r="AE3" s="3" t="n">
+      <c r="AG3" s="3" t="n">
         <v>10226036</v>
       </c>
-      <c r="AF3" s="3" t="n">
+      <c r="AH3" s="3" t="n">
         <v>296417</v>
       </c>
-      <c r="AG3" s="3" t="n">
+      <c r="AI3" s="3" t="n">
         <v>1470</v>
       </c>
-      <c r="AH3" s="3" t="n">
+      <c r="AJ3" s="3" t="n">
         <v>294947</v>
       </c>
-      <c r="AI3" s="3" t="n">
+      <c r="AK3" s="3" t="n">
         <v>423008</v>
       </c>
-      <c r="AJ3" s="3" t="n">
+      <c r="AL3" s="3" t="n">
         <v>2372</v>
       </c>
-      <c r="AK3" s="3" t="n">
+      <c r="AM3" s="3" t="n">
         <v>420636</v>
       </c>
     </row>
@@ -1005,30 +1035,36 @@
         <v>232938693</v>
       </c>
       <c r="AC4" s="3" t="n">
+        <v>232938693</v>
+      </c>
+      <c r="AD4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="3" t="n">
         <v>9356342</v>
       </c>
-      <c r="AD4" s="3" t="n">
+      <c r="AF4" s="3" t="n">
         <v>48178</v>
       </c>
-      <c r="AE4" s="3" t="n">
+      <c r="AG4" s="3" t="n">
         <v>9308164</v>
       </c>
-      <c r="AF4" s="3" t="n">
+      <c r="AH4" s="3" t="n">
         <v>40714</v>
       </c>
-      <c r="AG4" s="3" t="n">
+      <c r="AI4" s="3" t="n">
         <v>295</v>
       </c>
-      <c r="AH4" s="3" t="n">
+      <c r="AJ4" s="3" t="n">
         <v>40419</v>
       </c>
-      <c r="AI4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ4" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="AK4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM4" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1120,19 +1156,19 @@
         <v>241110478</v>
       </c>
       <c r="AC5" s="3" t="n">
+        <v>241110478</v>
+      </c>
+      <c r="AD5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="3" t="n">
         <v>9215588</v>
       </c>
-      <c r="AD5" s="3" t="n">
+      <c r="AF5" s="3" t="n">
         <v>49027</v>
       </c>
-      <c r="AE5" s="3" t="n">
+      <c r="AG5" s="3" t="n">
         <v>9166561</v>
-      </c>
-      <c r="AF5" s="3" t="n">
-        <v>10709</v>
-      </c>
-      <c r="AG5" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AH5" s="3" t="n">
         <v>10709</v>
@@ -1141,9 +1177,15 @@
         <v>0</v>
       </c>
       <c r="AJ5" s="3" t="n">
-        <v>0</v>
+        <v>10709</v>
       </c>
       <c r="AK5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1235,30 +1277,36 @@
         <v>237169533</v>
       </c>
       <c r="AC6" s="3" t="n">
+        <v>237169533</v>
+      </c>
+      <c r="AD6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="3" t="n">
         <v>10273319</v>
       </c>
-      <c r="AD6" s="3" t="n">
+      <c r="AF6" s="3" t="n">
         <v>57226</v>
       </c>
-      <c r="AE6" s="3" t="n">
+      <c r="AG6" s="3" t="n">
         <v>10216093</v>
       </c>
-      <c r="AF6" s="3" t="n">
+      <c r="AH6" s="3" t="n">
         <v>395162</v>
       </c>
-      <c r="AG6" s="3" t="n">
+      <c r="AI6" s="3" t="n">
         <v>2226</v>
       </c>
-      <c r="AH6" s="3" t="n">
+      <c r="AJ6" s="3" t="n">
         <v>392936</v>
       </c>
-      <c r="AI6" s="3" t="n">
+      <c r="AK6" s="3" t="n">
         <v>2113336</v>
       </c>
-      <c r="AJ6" s="3" t="n">
+      <c r="AL6" s="3" t="n">
         <v>13407</v>
       </c>
-      <c r="AK6" s="3" t="n">
+      <c r="AM6" s="3" t="n">
         <v>2099929</v>
       </c>
     </row>
@@ -1350,30 +1398,36 @@
         <v>240491977</v>
       </c>
       <c r="AC7" s="3" t="n">
+        <v>240491977</v>
+      </c>
+      <c r="AD7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="3" t="n">
         <v>9037742</v>
       </c>
-      <c r="AD7" s="3" t="n">
+      <c r="AF7" s="3" t="n">
         <v>49337</v>
       </c>
-      <c r="AE7" s="3" t="n">
+      <c r="AG7" s="3" t="n">
         <v>8988405</v>
       </c>
-      <c r="AF7" s="3" t="n">
+      <c r="AH7" s="3" t="n">
         <v>37824</v>
       </c>
-      <c r="AG7" s="3" t="n">
+      <c r="AI7" s="3" t="n">
         <v>124</v>
       </c>
-      <c r="AH7" s="3" t="n">
+      <c r="AJ7" s="3" t="n">
         <v>37700</v>
       </c>
-      <c r="AI7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ7" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="AK7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM7" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1465,30 +1519,36 @@
         <v>242265868</v>
       </c>
       <c r="AC8" s="3" t="n">
+        <v>242265868</v>
+      </c>
+      <c r="AD8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="3" t="n">
         <v>11096958</v>
       </c>
-      <c r="AD8" s="3" t="n">
+      <c r="AF8" s="3" t="n">
         <v>1021</v>
       </c>
-      <c r="AE8" s="3" t="n">
+      <c r="AG8" s="3" t="n">
         <v>11095937</v>
       </c>
-      <c r="AF8" s="3" t="n">
+      <c r="AH8" s="3" t="n">
         <v>894289</v>
       </c>
-      <c r="AG8" s="3" t="n">
+      <c r="AI8" s="3" t="n">
         <v>799</v>
       </c>
-      <c r="AH8" s="3" t="n">
+      <c r="AJ8" s="3" t="n">
         <v>893490</v>
       </c>
-      <c r="AI8" s="3" t="n">
+      <c r="AK8" s="3" t="n">
         <v>2070171</v>
       </c>
-      <c r="AJ8" s="3" t="n">
+      <c r="AL8" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="AK8" s="3" t="n">
+      <c r="AM8" s="3" t="n">
         <v>2070071</v>
       </c>
     </row>
@@ -1580,30 +1640,36 @@
         <v>239690178</v>
       </c>
       <c r="AC9" s="3" t="n">
+        <v>239690178</v>
+      </c>
+      <c r="AD9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="3" t="n">
         <v>9933729</v>
       </c>
-      <c r="AD9" s="3" t="n">
+      <c r="AF9" s="3" t="n">
         <v>58087</v>
       </c>
-      <c r="AE9" s="3" t="n">
+      <c r="AG9" s="3" t="n">
         <v>9875642</v>
       </c>
-      <c r="AF9" s="3" t="n">
+      <c r="AH9" s="3" t="n">
         <v>208710</v>
       </c>
-      <c r="AG9" s="3" t="n">
+      <c r="AI9" s="3" t="n">
         <v>1155</v>
       </c>
-      <c r="AH9" s="3" t="n">
+      <c r="AJ9" s="3" t="n">
         <v>207555</v>
       </c>
-      <c r="AI9" s="3" t="n">
+      <c r="AK9" s="3" t="n">
         <v>82054</v>
       </c>
-      <c r="AJ9" s="3" t="n">
+      <c r="AL9" s="3" t="n">
         <v>550</v>
       </c>
-      <c r="AK9" s="3" t="n">
+      <c r="AM9" s="3" t="n">
         <v>81504</v>
       </c>
     </row>
@@ -1695,30 +1761,36 @@
         <v>256903785</v>
       </c>
       <c r="AC10" s="3" t="n">
+        <v>256903785</v>
+      </c>
+      <c r="AD10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="3" t="n">
         <v>9976679</v>
       </c>
-      <c r="AD10" s="3" t="n">
+      <c r="AF10" s="3" t="n">
         <v>58506</v>
       </c>
-      <c r="AE10" s="3" t="n">
+      <c r="AG10" s="3" t="n">
         <v>9918173</v>
       </c>
-      <c r="AF10" s="3" t="n">
+      <c r="AH10" s="3" t="n">
         <v>736171</v>
       </c>
-      <c r="AG10" s="3" t="n">
+      <c r="AI10" s="3" t="n">
         <v>4593</v>
       </c>
-      <c r="AH10" s="3" t="n">
+      <c r="AJ10" s="3" t="n">
         <v>731578</v>
       </c>
-      <c r="AI10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ10" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="AK10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM10" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1810,30 +1882,36 @@
         <v>259488916</v>
       </c>
       <c r="AC11" s="3" t="n">
+        <v>259488916</v>
+      </c>
+      <c r="AD11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" s="3" t="n">
         <v>10871491</v>
       </c>
-      <c r="AD11" s="3" t="n">
+      <c r="AF11" s="3" t="n">
         <v>62410</v>
       </c>
-      <c r="AE11" s="3" t="n">
+      <c r="AG11" s="3" t="n">
         <v>10809081</v>
       </c>
-      <c r="AF11" s="3" t="n">
+      <c r="AH11" s="3" t="n">
         <v>308795</v>
       </c>
-      <c r="AG11" s="3" t="n">
+      <c r="AI11" s="3" t="n">
         <v>2021</v>
       </c>
-      <c r="AH11" s="3" t="n">
+      <c r="AJ11" s="3" t="n">
         <v>306774</v>
       </c>
-      <c r="AI11" s="3" t="n">
+      <c r="AK11" s="3" t="n">
         <v>2209831</v>
       </c>
-      <c r="AJ11" s="3" t="n">
+      <c r="AL11" s="3" t="n">
         <v>13586</v>
       </c>
-      <c r="AK11" s="3" t="n">
+      <c r="AM11" s="3" t="n">
         <v>2196245</v>
       </c>
     </row>
@@ -1925,30 +2003,36 @@
         <v>257607690</v>
       </c>
       <c r="AC12" s="3" t="n">
+        <v>257607690</v>
+      </c>
+      <c r="AD12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="3" t="n">
         <v>9031192</v>
       </c>
-      <c r="AD12" s="3" t="n">
+      <c r="AF12" s="3" t="n">
         <v>52409</v>
       </c>
-      <c r="AE12" s="3" t="n">
+      <c r="AG12" s="3" t="n">
         <v>8978783</v>
       </c>
-      <c r="AF12" s="3" t="n">
+      <c r="AH12" s="3" t="n">
         <v>15441</v>
       </c>
-      <c r="AG12" s="3" t="n">
+      <c r="AI12" s="3" t="n">
         <v>127</v>
       </c>
-      <c r="AH12" s="3" t="n">
+      <c r="AJ12" s="3" t="n">
         <v>15314</v>
       </c>
-      <c r="AI12" s="3" t="n">
+      <c r="AK12" s="3" t="n">
         <v>245590</v>
       </c>
-      <c r="AJ12" s="3" t="n">
+      <c r="AL12" s="3" t="n">
         <v>1680</v>
       </c>
-      <c r="AK12" s="3" t="n">
+      <c r="AM12" s="3" t="n">
         <v>243910</v>
       </c>
     </row>
@@ -2040,145 +2124,157 @@
         <v>263530256</v>
       </c>
       <c r="AC13" s="3" t="n">
+        <v>263530256</v>
+      </c>
+      <c r="AD13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="3" t="n">
         <v>10721231</v>
       </c>
-      <c r="AD13" s="3" t="n">
+      <c r="AF13" s="3" t="n">
         <v>58791</v>
       </c>
-      <c r="AE13" s="3" t="n">
+      <c r="AG13" s="3" t="n">
         <v>10662440</v>
       </c>
-      <c r="AF13" s="3" t="n">
+      <c r="AH13" s="3" t="n">
         <v>859215</v>
       </c>
-      <c r="AG13" s="3" t="n">
+      <c r="AI13" s="3" t="n">
         <v>5277</v>
       </c>
-      <c r="AH13" s="3" t="n">
+      <c r="AJ13" s="3" t="n">
         <v>853938</v>
-      </c>
-      <c r="AI13" s="3" t="n">
-        <v>3973</v>
-      </c>
-      <c r="AJ13" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AK13" s="3" t="n">
         <v>3973</v>
       </c>
+      <c r="AL13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM13" s="3" t="n">
+        <v>3973</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>TOTAL FY 2025-26</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="5" t="n">
         <v>235077</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="6" t="n">
         <v>4376552661</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="6" t="n">
         <v>3766866692.7</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="6" t="n">
         <v>291758299</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="6" t="n">
         <v>18465975</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="6" t="n">
         <v>8433197.5</v>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="6" t="n">
         <v>1541831.25</v>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="I14" s="6" t="n">
         <v>54964</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="J14" s="6" t="n">
         <v>22179195</v>
       </c>
-      <c r="K14" s="5" t="n">
+      <c r="K14" s="6" t="n">
         <v>554940</v>
       </c>
-      <c r="L14" s="5" t="n">
+      <c r="L14" s="6" t="n">
         <v>1726880</v>
       </c>
-      <c r="M14" s="5" t="n">
+      <c r="M14" s="6" t="n">
         <v>18992776</v>
       </c>
-      <c r="N14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="5" t="n">
+      <c r="N14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="6" t="n">
         <v>153429</v>
       </c>
-      <c r="Q14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="5" t="n">
+      <c r="Q14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="6" t="n">
         <v>511757</v>
       </c>
-      <c r="T14" s="5" t="n">
+      <c r="T14" s="6" t="n">
         <v>316207</v>
       </c>
-      <c r="U14" s="5" t="n">
+      <c r="U14" s="6" t="n">
         <v>6692144</v>
       </c>
-      <c r="V14" s="5" t="n">
+      <c r="V14" s="6" t="n">
         <v>263784</v>
       </c>
-      <c r="W14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="5" t="n">
+      <c r="W14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="6" t="n">
         <v>1155540087.39</v>
       </c>
-      <c r="AA14" s="5" t="n">
+      <c r="AA14" s="6" t="n">
         <v>1443565363.97</v>
       </c>
-      <c r="AB14" s="5" t="n">
+      <c r="AB14" s="6" t="n">
         <v>2932989494</v>
       </c>
-      <c r="AC14" s="5" t="n">
+      <c r="AC14" s="6" t="n">
+        <v>2932989494</v>
+      </c>
+      <c r="AD14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="6" t="n">
         <v>118459584</v>
       </c>
-      <c r="AD14" s="5" t="n">
+      <c r="AF14" s="6" t="n">
         <v>604819</v>
       </c>
-      <c r="AE14" s="5" t="n">
+      <c r="AG14" s="6" t="n">
         <v>117854765</v>
       </c>
-      <c r="AF14" s="5" t="n">
+      <c r="AH14" s="6" t="n">
         <v>4183925</v>
       </c>
-      <c r="AG14" s="5" t="n">
+      <c r="AI14" s="6" t="n">
         <v>20140</v>
       </c>
-      <c r="AH14" s="5" t="n">
+      <c r="AJ14" s="6" t="n">
         <v>4163785</v>
       </c>
-      <c r="AI14" s="5" t="n">
+      <c r="AK14" s="6" t="n">
         <v>7147963</v>
       </c>
-      <c r="AJ14" s="5" t="n">
+      <c r="AL14" s="6" t="n">
         <v>31695</v>
       </c>
-      <c r="AK14" s="5" t="n">
+      <c r="AM14" s="6" t="n">
         <v>7116268</v>
       </c>
     </row>
@@ -61929,7 +62025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -62027,43 +62123,50 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Checks: REVISED GROSS - REVISED TOTAL DEDUCTION vs REVISED NET PAYABLE; monthly diff is within ~Rs.365</t>
+          <t>Original NETPAYABLE vs REVISED NET PAYABLE: exactly Rs.0 every month (golden rule - net payable never changes).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>(stored-value rounding, consistent with the C2 tolerance in the reconciliation skill).</t>
+          <t>Checks: REVISED GROSS - REVISED TOTAL DEDUCTION vs REVISED NET PAYABLE; monthly diff is within ~Rs.365</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Verification: REVISED PF and REVISED NET PAYABLE totals for all 12 months match the PF_ESI_Reco_Summary</t>
+          <t>(stored-value rounding, consistent with the C2 tolerance in the reconciliation skill).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Verification: REVISED PF and REVISED NET PAYABLE totals for all 12 months match the PF_ESI_Reco_Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>file produced earlier today (11-Jul-2026) in this same folder.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Full per-column sums for every month (AllColumns_Detail) are in the audit workbook in the GitHub repo</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
+        <is>
+          <t>Full per-column sums for every month (AllColumns_Detail) are in the audit workbook in the GitHub repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>anthropic-finance (docs/salary-monthly-summary-fy2025-26/).</t>
         </is>

</xml_diff>